<commit_message>
scan: seg5 2026-10-14 00:57 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-10-13.xlsx
+++ b/output/full_scan/batch_seq6_2026-10-13.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>64.464862835139</v>
+        <v>64.46486284747294</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>15.14040890687835</v>
+        <v>15.14040883977694</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>3.979106860235433</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1.679349676028586</v>
+        <v>1.679349675836324</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>64.43175472567179</v>
+        <v>64.43175474398919</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>20.7512085106803</v>
+        <v>20.7512085683774</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>3.694930975308025</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.4166074362802153</v>
+        <v>0.4166074362081124</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>62.95837792849377</v>
+        <v>62.95837804299673</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>35.50654379782672</v>
+        <v>35.50654386598853</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>1.452825304547327</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>-0.2598155961159269</v>
+        <v>-0.2598155967408315</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>67.85634075310406</v>
+        <v>67.85634079828705</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>39.14569722085954</v>
+        <v>39.14569742469243</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>1.646585532546797</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.8529602560448377</v>
+        <v>0.8529602558886071</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>75.10900500815353</v>
+        <v>75.10900502290397</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>40.21283872643129</v>
+        <v>40.21283881402295</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>3.603345930101358</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>5.66020992756264</v>
+        <v>5.660209927322303</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>61.61502637410852</v>
+        <v>61.61502644804351</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>29.63347005235405</v>
+        <v>29.63346997543648</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.610038591883432</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>5.625322358616998</v>
+        <v>5.625322357415236</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>57.97427556799769</v>
+        <v>57.97427575246923</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>32.68441727359992</v>
+        <v>32.68441748761051</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.825269320344595</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.0034593076249334</v>
+        <v>0.0034593070961781</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>65.73587621256902</v>
+        <v>65.73587629111648</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>24.80837990382178</v>
+        <v>24.80837989689453</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>4.828695950678907</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.5861682444586784</v>
+        <v>0.5861682441221974</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -951,21 +951,21 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6271</v>
+        <v>6438</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>同欣電</t>
+          <t>迅得</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1015.69183459794</v>
+        <v>1018.039472346988</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>240</v>
+        <v>176.5</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,49 +976,49 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>60.50410230263328</v>
+        <v>75.14583299166982</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>29.30326538027049</v>
+        <v>36.53539710298829</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1.832653909821332</v>
+        <v>3.903947234698799</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M10" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.6895635082910987</v>
+        <v>1.60315023872201</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>6191</v>
+        <v>6271</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>精成科</t>
+          <t>同欣電</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>984</v>
+        <v>1015.69183459794</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>96.40000000000001</v>
+        <v>240</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,49 +1029,49 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>80.44598559043808</v>
+        <v>60.50410236564522</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>26.5335388770509</v>
+        <v>29.30326544993911</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>7.918070534255429</v>
+        <v>1.832653909821332</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>1.370451270943915</v>
+        <v>0.6895635080507754</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>6438</v>
+        <v>6191</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>迅得</t>
+          <t>精成科</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>958.039472346988</v>
+        <v>984</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>176.5</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,25 +1082,25 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>75.14583265018727</v>
+        <v>80.4459859310509</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>36.53539696888628</v>
+        <v>26.53353885477089</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>3.903947234698799</v>
+        <v>7.918070534255429</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>1.603150240885135</v>
+        <v>1.370451269982546</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>67.64679295192124</v>
+        <v>67.64679298292526</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>37.85312236147498</v>
+        <v>37.85312259823593</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.8520425661008714</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>3.256672434314696</v>
+        <v>3.256672433737862</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>906.4830597587852</v>
+        <v>906.4830597587816</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>49.5</v>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>56.94873401035524</v>
+        <v>56.94873423037413</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>22.26090895887159</v>
+        <v>22.26090896334004</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.7442866289677921</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.0463603329584217</v>
+        <v>0.046360332742118</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>61.92463684501996</v>
+        <v>61.92463689347139</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>18.06021202521456</v>
+        <v>18.06021210687004</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>2.412182653048067</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.4656554565732219</v>
+        <v>0.4656554564770886</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>53.21013800302235</v>
+        <v>53.21013801854231</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>22.01237618755102</v>
+        <v>22.01237625391444</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>2.571376696177176</v>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>77.29537726043874</v>
+        <v>77.29537736130197</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>30.26043611422533</v>
+        <v>30.26043612445929</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.524657700327506</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.2646766339489068</v>
+        <v>0.2646766338888229</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>60.62773815892144</v>
+        <v>60.62773815938258</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>48.11914843832555</v>
+        <v>48.1191484014096</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.6491797818917961</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.6774463407755231</v>
+        <v>-0.6774463407923488</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>70.79835191078243</v>
+        <v>70.79835209968419</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>25.37105888989459</v>
+        <v>25.37105904925764</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.4301134489841777</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-0.6402494116485471</v>
+        <v>-0.6402494120090436</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>856.4887611597848</v>
+        <v>856.4887611597852</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1600</v>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>67.70632342865049</v>
+        <v>67.70632346741498</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>30.4184166036821</v>
+        <v>30.41841675630065</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>2.321741749558652</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>35.93817167161956</v>
+        <v>35.93817166669248</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>60.09368130586886</v>
+        <v>60.09368168110999</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>23.74817023786372</v>
+        <v>23.74817038129011</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.014801423433367</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.08833255456116069</v>
+        <v>0.0883325542967769</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>67.11498471827554</v>
+        <v>67.11498479532446</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>41.00907912608943</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>1.759698839152959</v>
+        <v>1.75969883888857</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>67.59581100577179</v>
+        <v>67.59581125805627</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>21.85952129951379</v>
+        <v>21.85952127225872</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>4.6724577413294</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.1378186142253191</v>
+        <v>0.1378186141652327</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>805.4913560233014</v>
+        <v>805.4913560233008</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>641</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>64.07794928867662</v>
+        <v>64.07794937407178</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>37.94965670499796</v>
+        <v>37.94965671581154</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.630288778487762</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>7.744872810713499</v>
+        <v>7.744872808310063</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>58.89923314520295</v>
+        <v>58.89923332503795</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>28.49507975358992</v>
+        <v>28.49507977383916</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.717419672759461</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.9517552651714988</v>
+        <v>0.9517552649311528</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>70.23970191040137</v>
+        <v>70.23970189390207</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>24.81594058611012</v>
+        <v>24.81594060911958</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.6863344954638941</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.55411978210526</v>
+        <v>1.554119782369639</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>778.1801878027394</v>
+        <v>778.1801878027395</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>173</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>61.60210863935799</v>
+        <v>61.6021087287849</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>28.19199160825801</v>
+        <v>28.1919915812065</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.167101547499344</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>1.74020160021276</v>
+        <v>1.7402015996119</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>763.4080697663899</v>
+        <v>763.4080697663895</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>1655</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>58.70604162233964</v>
+        <v>58.70604166017001</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>24.3942833255714</v>
+        <v>24.39428344340159</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>1.036855683960017</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>22.18347682603405</v>
+        <v>22.18347682110696</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>55.77498672271699</v>
+        <v>55.77498681694699</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>17.36728311420217</v>
+        <v>17.36728314764541</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.8187564347463054</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>3.190576248697758</v>
+        <v>3.190576248096904</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>67.44180172669721</v>
+        <v>67.44180173194474</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>23.42713283230458</v>
+        <v>23.42713286224729</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>2.654382457269053</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>7.172143386421212</v>
+        <v>7.172143389545695</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>50.14137455421139</v>
+        <v>50.14137461816485</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>31.11160246154889</v>
+        <v>31.11160248163724</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.3860228591752059</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.190631966156759</v>
+        <v>-0.1906319664451636</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>682.4292592641771</v>
+        <v>682.4292592641767</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>25.1</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>80.5072145928083</v>
+        <v>80.50721473280663</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>40.5205926005197</v>
+        <v>40.52059271408626</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.256792417155118</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.3819475124354721</v>
+        <v>0.3819475123513454</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>681.2996083819975</v>
+        <v>681.2996083819974</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>45.7</v>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>76.59946460906099</v>
+        <v>76.59946477747864</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>24.5545628595634</v>
+        <v>24.55456287001974</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>1.445819053270903</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.3049523936988729</v>
+        <v>0.3049523935787014</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>60.58548650305929</v>
+        <v>60.58548650591644</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>25.85667661942274</v>
+        <v>25.8566766480125</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.324423946763004</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1.431573374153813</v>
+        <v>1.431573374117759</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>666.9210358804802</v>
+        <v>666.921035880478</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>73.90000000000001</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>57.54520399180154</v>
+        <v>57.54520393657067</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>25.03386458608651</v>
+        <v>25.03386467567827</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6728779703625287</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.5533182355161972</v>
+        <v>0.5533182352998847</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>644.9724522974121</v>
+        <v>644.9724522974124</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>296</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>53.23555143084587</v>
+        <v>53.23555149469165</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>18.24243925537608</v>
+        <v>18.24243955326346</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.8121640428346091</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>1.063990169887627</v>
+        <v>1.063990169046396</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>42.23964973142976</v>
+        <v>42.23964975565092</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>38.85332340510392</v>
+        <v>38.8533234816035</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.5975203059971422</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-1.271495554211914</v>
+        <v>-1.27149555469261</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>58.10527225100507</v>
+        <v>58.10527229263219</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>31.18947589749195</v>
+        <v>31.18947593568833</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.8254201694429805</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.072178281964268</v>
+        <v>0.07217828179604339</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>633.3137561403017</v>
+        <v>633.3137561403023</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>74.2</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>50.91236202312132</v>
+        <v>50.91236211177092</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>21.0982710097828</v>
+        <v>21.0982711556722</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.5932512381745694</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.77595648148053</v>
+        <v>0.775956481107989</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>54.9270439536006</v>
+        <v>54.92704394687355</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>33.4647770387493</v>
+        <v>33.46477694974197</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.4509952090399809</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.2647085864042964</v>
+        <v>0.2647085865965675</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>48.40966822043509</v>
+        <v>48.40966824166765</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>38.16118727294087</v>
+        <v>38.16118739418962</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.7585810915169089</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-1.689630415707101</v>
+        <v>-1.689630415911398</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>47.70102931548985</v>
+        <v>47.70102935655372</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>47.73289348049585</v>
+        <v>47.73289360500993</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.3544016780080934</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-1.056043500837909</v>
+        <v>-1.056043500934051</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>51.81417152122676</v>
+        <v>51.81417153684985</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>38.46113757511654</v>
+        <v>38.46113778806465</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.2894454963500344</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-4.757904489102373</v>
+        <v>-4.757904489445735</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>50.22920074416987</v>
+        <v>50.22920075161314</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>33.69503825961333</v>
+        <v>33.69503824082958</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.6532695560044951</v>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>611.4387160642651</v>
+        <v>611.4387160642647</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>5940</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>57.33683810394204</v>
+        <v>57.3368381664759</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>13.56877695531467</v>
+        <v>13.56877732787049</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.525817033198133</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>77.7948050489677</v>
+        <v>77.79480502012643</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>63.68745206615328</v>
+        <v>63.6874520932093</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>13.77130598881731</v>
+        <v>13.771305993836</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>8.057819632048583</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.6244263029700542</v>
+        <v>0.6244263028979575</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>600.0927550191224</v>
+        <v>600.092755019123</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>113</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>53.97089881734536</v>
+        <v>53.97089910206576</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>26.35389972197833</v>
+        <v>26.35389975748567</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.8400096351775838</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.5544167716556883</v>
+        <v>0.5544167711749839</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>591.8629041551536</v>
+        <v>591.862904155153</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>49</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>47.18404514571784</v>
+        <v>47.18404523900964</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>8.642415895056567</v>
+        <v>8.642415977308731</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>4.199462998705999</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.0075523853166696</v>
+        <v>-0.0075523854728961</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>53.19810295545622</v>
+        <v>53.19810296516014</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>4.60485662531466</v>
+        <v>4.604856743730593</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>3.999902960271562</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.1324593979973812</v>
+        <v>0.132459397949312</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3099,7 +3099,7 @@
         <v>56.02680445028442</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>14.9618201849408</v>
+        <v>14.96182022327598</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>2.73999412858401</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.4321202240448161</v>
+        <v>-0.4321202238645565</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>575.2301463579473</v>
+        <v>575.2301463579479</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>63.2</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>47.42777299912886</v>
+        <v>47.42777351682685</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>26.11964171850517</v>
+        <v>26.11964165232789</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>1.962010861481348</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.5115185362445043</v>
+        <v>0.5115185348024334</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>50.93232794964438</v>
+        <v>50.93232798418202</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>29.88954949325467</v>
+        <v>29.88954951686391</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.2817661361495195</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.675000798115746</v>
+        <v>0.675000797947515</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>562.1029838495278</v>
+        <v>562.1029838495306</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>43.6</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>48.04520902408397</v>
+        <v>48.04520910933689</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>17.89726537231713</v>
+        <v>17.89726553284675</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>2.256352564160143</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.2660667726623932</v>
+        <v>0.2660667724701138</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>60.16954232480177</v>
+        <v>60.16954235521507</v>
       </c>
       <c r="I54" s="2" t="n">
         <v>31.48030612321612</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.1755983612084287</v>
+        <v>0.175598361184398</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>54.2208189316789</v>
+        <v>54.22081895232762</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>35.08399629784423</v>
+        <v>35.08399636006222</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.7801798274371343</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.1590999919109501</v>
+        <v>-0.1590999920912106</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>41.39238264917689</v>
+        <v>41.3923826738325</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>26.75275017177794</v>
+        <v>26.75275016795779</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.5346400859019071</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-1.393230096972419</v>
+        <v>-1.393230097308898</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>49.11900999659196</v>
+        <v>49.11901025637002</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>30.5203597185441</v>
+        <v>30.52035978037873</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.000914677858621</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.2599385786317001</v>
+        <v>-0.2599385851210726</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>47.55776352500251</v>
+        <v>47.55776358472788</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>29.89244114683114</v>
+        <v>29.89244123747309</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.930956253606992</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-1.863153335092242</v>
+        <v>-1.86315333593346</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>38.83217109544049</v>
+        <v>38.83217116236504</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>23.78210449631149</v>
+        <v>23.78210478186151</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1.000917471125347</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.8100065247547161</v>
+        <v>-0.8100065259564468</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>53.60668729181763</v>
+        <v>53.6066873117666</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>21.16190718277926</v>
+        <v>21.16190718601897</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.162622615040778</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.8817159056571362</v>
+        <v>0.8817159056331021</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>52.91335601152191</v>
+        <v>52.913356008967</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>7.932121199327515</v>
+        <v>7.932121132100925</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>1.843141771277208</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.7388632694140764</v>
+        <v>0.738863269510215</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>47.85730913709202</v>
+        <v>47.8573092558625</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>13.36600394749382</v>
+        <v>13.36600400504731</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>1.07322160537594</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.4152860096325825</v>
+        <v>-0.4152860099931156</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>509.7111503446569</v>
+        <v>509.7111503446578</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>50.8</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>42.14171322658679</v>
+        <v>42.14171326367165</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>8.884646551576493</v>
+        <v>8.884646532064529</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.8508275470721993</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0030975815803948</v>
+        <v>0.0030975815563688</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>42.94388121850123</v>
+        <v>42.943881296123</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>16.71256347121447</v>
+        <v>16.71256352988926</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.8379394904327317</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.1090752068962799</v>
+        <v>-0.1090752070404892</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>45.86315047169001</v>
+        <v>45.86315054823916</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>8.977162876840902</v>
+        <v>8.977162518043126</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.7684259625164387</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.3025917314813067</v>
+        <v>0.3025917312959547</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>42.93705292832078</v>
+        <v>42.93705308105352</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>7.511414434758248</v>
+        <v>7.511414524324795</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.78310968098348</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.0805110350348551</v>
+        <v>-0.0805110353953781</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>41.73941135865734</v>
+        <v>41.73941134763782</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>14.18616530690541</v>
+        <v>14.18616532050871</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4121389422845233</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>4.409333796902217</v>
+        <v>4.409333797503024</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>481.2828801213304</v>
+        <v>481.2828801213305</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>91.59999999999999</v>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>49.67323127419158</v>
+        <v>49.67323152732035</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>8.522618135467074</v>
+        <v>8.522618389471836</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>2.494639929373187</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.0485658050864555</v>
+        <v>0.0485658049422404</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>48.37430360122445</v>
+        <v>48.37430380551413</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>15.013689088412</v>
+        <v>15.01368911393524</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1.208695987167166</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>3.311481382969895</v>
+        <v>3.311481378162973</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>44.25057878389827</v>
+        <v>44.25057881141034</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>13.2063390659239</v>
+        <v>13.20633908260034</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.2275944099019429</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.1303265944475429</v>
+        <v>-0.1303265947119203</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>459.8451834324239</v>
+        <v>459.8451834324235</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>33.35</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>41.74937884828327</v>
+        <v>41.74937947518957</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>28.01707112226982</v>
+        <v>28.01707134735069</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>1.321718489578157</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.2054454298866709</v>
+        <v>-0.205445430427449</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>47.30938065000414</v>
+        <v>47.30938077386351</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>22.38083436924575</v>
+        <v>22.38083447759443</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.4519455231105425</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0202882883403306</v>
+        <v>0.0202882882201534</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>454.3965346479022</v>
+        <v>454.3965346479023</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>25.1</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>39.83480657526688</v>
+        <v>39.83480659643747</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>15.61208740274793</v>
+        <v>15.61208739453778</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>2.545414853284818</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.0646036455517416</v>
+        <v>0.06460364557577999</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>51.89556019479944</v>
+        <v>51.8955601708486</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>21.21073966602243</v>
+        <v>21.21073992528258</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.4115077747812148</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.2629357971838515</v>
+        <v>0.2629357970756981</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>446.5110364898198</v>
+        <v>446.5110364898214</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>20.2</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>52.54512475019568</v>
+        <v>52.54512477635802</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>7.20844356194478</v>
+        <v>7.208443490343199</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.3724360108378879</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.3982193310527551</v>
+        <v>0.3982193308364449</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>434.7919858821268</v>
+        <v>434.7919858821267</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>83.7</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>46.22661253652849</v>
+        <v>46.22661255723224</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>23.95048049499753</v>
+        <v>23.95048053381008</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.5036466956015929</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.5171351052742716</v>
+        <v>-0.5171351058510925</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>46.61781125330275</v>
+        <v>46.61781128460376</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>23.95041510254059</v>
+        <v>23.95041527016551</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.6093146821119882</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.4383419286200292</v>
+        <v>-0.4383419288003036</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>421.102602875426</v>
+        <v>421.1026028754254</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>110.5</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>47.03529899702733</v>
+        <v>47.03529957090389</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>18.51376989047263</v>
+        <v>18.5137699967163</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.6650397833019611</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.0622038012395667</v>
+        <v>0.0622037993167871</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>411.8479225029491</v>
+        <v>411.8479225029492</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>46</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>44.61882020100494</v>
+        <v>44.61882028803883</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>13.13978105676783</v>
+        <v>13.13978109715368</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.5114528414603945</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.022122867157641</v>
+        <v>-0.0221228673018486</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>45.67044626978286</v>
+        <v>45.67044682114662</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>11.46386086885077</v>
+        <v>11.46386099021848</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>1.011653106811299</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.3261877091324114</v>
+        <v>-0.3261877095443167</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>394.5992192439815</v>
+        <v>394.5992192439834</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>25.35</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>42.53257149834864</v>
+        <v>42.53257150945608</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>26.46728522922841</v>
+        <v>26.46728521542317</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.4530725293369823</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.1320302477624361</v>
+        <v>-0.1320302478345408</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>393.7717373126067</v>
+        <v>393.7717373126068</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>854</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>35.83500418839385</v>
+        <v>35.83500439492995</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>13.2707546774589</v>
+        <v>13.27075463648476</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>1.18110276362141</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>1.279789058683633</v>
+        <v>1.279789055318812</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
         <v>41.49096370568289</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>32.89560133634078</v>
+        <v>32.89560134522993</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>1.286306567641388</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>36.56093251905856</v>
+        <v>36.56093258633714</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>23.85146466365002</v>
+        <v>23.85146489043447</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.4556595533838664</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-12.00321121803393</v>
+        <v>-12.00321122127862</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>37.67458340181727</v>
+        <v>37.67458343562367</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>17.14675284549624</v>
+        <v>17.14675301297251</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>1.035003312065398</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.07191779868404601</v>
+        <v>0.0719177985879044</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>374.3395421397109</v>
+        <v>374.339542139711</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>1630</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>50.67686659736717</v>
+        <v>50.67686663612848</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>21.10815727504554</v>
+        <v>21.10815733295597</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>1.435677452354706</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>14.85080437559695</v>
+        <v>14.8508043698285</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>48.17869584717025</v>
+        <v>48.17869586211078</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>25.98444147590046</v>
+        <v>25.9844415232289</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.3751647890434549</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.5308816191396339</v>
+        <v>0.5308816190314831</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>349.4880742333326</v>
+        <v>349.4880742333325</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>39.95</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>40.87833887206388</v>
+        <v>40.87833935309774</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>23.47359498579797</v>
+        <v>23.47359489645214</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.9718273109335968</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0440825550671439</v>
+        <v>0.044082554850825</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>48.41992557320005</v>
+        <v>48.41992571473339</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>17.41859882829822</v>
+        <v>17.41859894830499</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.592835306782732</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.2593276306611373</v>
+        <v>0.2593276304688638</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>38.82216399552048</v>
+        <v>38.8221643315517</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>15.19158436645541</v>
+        <v>15.1915843285145</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.7063682942085053</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.024990123500444</v>
+        <v>0.0249901232841311</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>45.56876865392371</v>
+        <v>45.56876876944156</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>16.56260575885536</v>
+        <v>16.56260579997112</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.9500889405577536</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.0120918588918847</v>
+        <v>0.0120918588197775</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>54.30821184711449</v>
+        <v>54.30821186920819</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>14.26176660243344</v>
+        <v>14.26176648882928</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.893053138803373</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.3944692007712183</v>
+        <v>0.3944692005428911</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>338.2677925797541</v>
+        <v>338.267792579754</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>12.4</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>40.45187717158344</v>
+        <v>40.45187827097476</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>17.95624867449338</v>
+        <v>17.95624869003603</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>1.331266824373929</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.036002822084515</v>
+        <v>-0.0360028221926721</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>46.35336522238351</v>
+        <v>46.35336565918646</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>30.67622575168491</v>
+        <v>30.67622585427243</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.6093834493808971</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.1086168631499807</v>
+        <v>-0.1086168633662922</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>36.88849145625985</v>
+        <v>36.88849150527152</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>8.41707205552607</v>
+        <v>8.417072242619417</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.623234810333611</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-2.258391771845539</v>
+        <v>-2.258391773768301</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>328.3838632066743</v>
+        <v>328.3838632066742</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>12.65</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>52.92767236738781</v>
+        <v>52.92767246519752</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>33.45981607476531</v>
+        <v>33.45981617617834</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.5339256516865203</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0488295373983076</v>
+        <v>0.0488295373502377</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>323.4744112284328</v>
+        <v>323.4744112284327</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>10.3</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>48.77258351304166</v>
+        <v>48.77258461517152</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>14.02569958205226</v>
+        <v>14.02569944602689</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.9922289282288724</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.0238215498526453</v>
+        <v>0.0238215497405659</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>43.99785735747107</v>
+        <v>43.99785751336507</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>22.13632857570785</v>
+        <v>22.13632860223806</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.4187135971244413</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.0489831508812028</v>
+        <v>-0.0489831510254102</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>39.49775773956056</v>
+        <v>39.49775786314424</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>19.61014305112303</v>
+        <v>19.61014311484675</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>1.317021423794479</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.0188002808014359</v>
+        <v>-0.0188002808975762</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>319.656427162789</v>
+        <v>319.6564271627891</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>97</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>40.33365681426437</v>
+        <v>40.33365687978912</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>18.20825198972941</v>
+        <v>18.20825198777396</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.8193049156066066</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.3747249361385212</v>
+        <v>-0.3747249366192179</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>40.41185070532707</v>
+        <v>40.41185081354298</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>11.95613334725102</v>
+        <v>11.9561335086971</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.8771367588646743</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.320911907167531</v>
+        <v>-0.3209119075040127</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>41.28321113421979</v>
+        <v>41.28321115090283</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>15.5197288432155</v>
+        <v>15.51972901817795</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.7848655508357726</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.2950691752945655</v>
+        <v>-0.2950691756310597</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>33.17199978346144</v>
+        <v>33.17200038666273</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>9.035931293583849</v>
+        <v>9.035931324368892</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>1.751347751718311</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0004629314501915</v>
+        <v>-0.0004629316665052</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>39.98351788135647</v>
+        <v>39.98351801585748</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>14.58129796171512</v>
+        <v>14.58129812013045</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.6394003871888299</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.0155878857576453</v>
+        <v>-0.0155878861542191</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>36.63984397765313</v>
+        <v>36.6398439814247</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>16.11653999627681</v>
+        <v>16.11654009388118</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.7330690922309046</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.4538880472521339</v>
+        <v>-0.4538880472641506</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>290.6181769803707</v>
+        <v>290.6181769803708</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>74.09999999999999</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>39.21170504792519</v>
+        <v>39.21170512167102</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.48670099784189</v>
+        <v>16.48670111376349</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>1.141376999895299</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.2000502456644001</v>
+        <v>0.2000502451837181</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>284.4108048500968</v>
+        <v>284.4108048500995</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>21.45</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>35.75567858996217</v>
+        <v>35.75567865446772</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>16.37114290027645</v>
+        <v>16.37114290125179</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>1.000036971465803</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.1614091673159287</v>
+        <v>-0.1614091675082059</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>39.82602539512743</v>
+        <v>39.82602542687558</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>14.55721926765793</v>
+        <v>14.55721928582041</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>1.226194646920568</v>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>246.4937840529001</v>
+        <v>246.4937840529003</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>18.5</v>
@@ -6226,7 +6226,7 @@
         <v>49.64761933284746</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>14.18288405412772</v>
+        <v>14.18288396648695</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>2.725659026223018</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.1987296833266868</v>
+        <v>0.1987296830863389</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6279,7 +6279,7 @@
         <v>33.52568357800885</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>18.50364948488888</v>
+        <v>18.5036494472051</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.9525896847666984</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>40.40376449557135</v>
+        <v>40.40376502696343</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>21.48377150956255</v>
+        <v>21.48377164982231</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.5683456841524265</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.2186563658538191</v>
+        <v>-0.2186563664066163</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>180.4631905230113</v>
+        <v>180.4631905230114</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>91.8</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>34.05040274974345</v>
+        <v>34.05040325233234</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>10.94100810506922</v>
+        <v>10.94100837120064</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>1.019721517942981</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.490021697117102</v>
+        <v>-0.4900217004819587</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>46.37604376756813</v>
+        <v>46.37604376154222</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>16.58221381498402</v>
+        <v>16.58221383189214</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.5907111963939439</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>37.40769829414855</v>
+        <v>37.4076984428048</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>18.69344601327693</v>
+        <v>18.69344601795864</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.839229567813741</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.207533080605251</v>
+        <v>-0.2075330808215658</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>93.6421605786894</v>
+        <v>93.64216057869056</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>35.6</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>30.80162457749597</v>
+        <v>30.80162478502585</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>17.61718378850502</v>
+        <v>17.61718371585655</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.9284359647675676</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.3392951132398236</v>
+        <v>-0.3392951133359605</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>

</xml_diff>